<commit_message>
Atualização automática portal convênios
</commit_message>
<xml_diff>
--- a/upload/pagamento2026.xlsx
+++ b/upload/pagamento2026.xlsx
@@ -1024,12 +1024,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>89045.45</t>
+          <t>178090.9</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>89045.45</t>
+          <t>178090.9</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -1285,12 +1285,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>63495.81</t>
+          <t>126991.62</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>63495.81</t>
+          <t>126991.62</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -3199,12 +3199,12 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>84912.15</t>
+          <t>169824.31</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>84912.15</t>
+          <t>169824.31</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
@@ -8158,12 +8158,12 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>608660.04</t>
+          <t>1217320.08</t>
         </is>
       </c>
       <c r="P89" s="2" t="inlineStr">
         <is>
-          <t>608660.04</t>
+          <t>1217320.08</t>
         </is>
       </c>
       <c r="Q89" s="2" t="inlineStr">
@@ -8245,12 +8245,12 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>566736.12</t>
+          <t>1133472.24</t>
         </is>
       </c>
       <c r="P90" s="2" t="inlineStr">
         <is>
-          <t>566736.12</t>
+          <t>1133472.24</t>
         </is>
       </c>
       <c r="Q90" s="2" t="inlineStr">
@@ -8332,12 +8332,12 @@
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>609610.92</t>
+          <t>1219221.84</t>
         </is>
       </c>
       <c r="P91" s="2" t="inlineStr">
         <is>
-          <t>609610.92</t>
+          <t>1219221.84</t>
         </is>
       </c>
       <c r="Q91" s="2" t="inlineStr">
@@ -10604,7 +10604,7 @@
       </c>
       <c r="Q117" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270000</t>
         </is>
       </c>
     </row>

</xml_diff>